<commit_message>
:white_circle: Dev v4.1.10: CH4 - CAPEX,OPEX,ROI (editing)
</commit_message>
<xml_diff>
--- a/02_Codigo/04_BattBankDesign/01_codes/01_Pnom015/CAPEX_OPEX_ROI_15.xlsx
+++ b/02_Codigo/04_BattBankDesign/01_codes/01_Pnom015/CAPEX_OPEX_ROI_15.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\desar\Documents\Tesis Magister\Tesis_Msc_LSZ\02_Codigo\04_BattBankDesign\01_codes\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\desar\Documents\Tesis Magister\Tesis_Msc_LSZ\02_Codigo\04_BattBankDesign\01_codes\01_Pnom015\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{700F1A8B-F0D9-49FF-BAA5-C4A69971324E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E270F721-9F6D-4A59-A1F3-D54E035396E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-11610" windowWidth="29040" windowHeight="15840" activeTab="5" xr2:uid="{32DAA168-B565-429F-AAFE-E289AA3DABBF}"/>
+    <workbookView xWindow="-28920" yWindow="-11610" windowWidth="29040" windowHeight="15840" activeTab="4" xr2:uid="{32DAA168-B565-429F-AAFE-E289AA3DABBF}"/>
   </bookViews>
   <sheets>
     <sheet name="Costs 15%" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="144" uniqueCount="71">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="162" uniqueCount="74">
   <si>
     <t>Lowest Cost ($/kWh)</t>
   </si>
@@ -254,6 +254,15 @@
   </si>
   <si>
     <t>Cost LTO</t>
+  </si>
+  <si>
+    <t>20 años</t>
+  </si>
+  <si>
+    <t>10 años</t>
+  </si>
+  <si>
+    <t>15 años</t>
   </si>
 </sst>
 </file>
@@ -1657,14 +1666,29 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D9148CD0-5187-4E9B-AB88-218957DBEFDE}">
-  <dimension ref="B2:L13"/>
+  <dimension ref="B1:O13"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="15.36328125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="9.08984375" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="11.26953125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="1" spans="2:15" x14ac:dyDescent="0.35">
+      <c r="H1" s="16" t="s">
+        <v>72</v>
+      </c>
+      <c r="I1" s="16"/>
+      <c r="K1" s="16" t="s">
+        <v>73</v>
+      </c>
+      <c r="L1" s="16"/>
+      <c r="N1" s="16" t="s">
+        <v>71</v>
+      </c>
+      <c r="O1" s="16"/>
+    </row>
+    <row r="2" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B2" t="s">
         <v>44</v>
       </c>
@@ -1682,17 +1706,30 @@
         <v>48</v>
       </c>
       <c r="I2" s="8">
-        <f>SUM(C9:L9)+SUM(C13:L13)-F2</f>
-        <v>2445271.9057673095</v>
-      </c>
-    </row>
-    <row r="3" spans="2:12" x14ac:dyDescent="0.35">
+        <f>SUM($C$9:$L$9)-F2</f>
+        <v>1153542.1213406175</v>
+      </c>
+      <c r="K2" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="L2" s="8">
+        <f>SUM($C$9:$L$9)+SUM($C$13:$G$13)-F2</f>
+        <v>2478158.13439776</v>
+      </c>
+      <c r="N2" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="O2" s="8">
+        <f>SUM($C$9:$L$9)+SUM($C$13:$L$13)-F2</f>
+        <v>3379669.5354062933</v>
+      </c>
+    </row>
+    <row r="3" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B3" t="s">
         <v>46</v>
       </c>
       <c r="C3" s="10">
-        <f>0.1</f>
-        <v>0.1</v>
+        <v>0.08</v>
       </c>
       <c r="E3" t="s">
         <v>69</v>
@@ -1705,11 +1742,25 @@
         <v>49</v>
       </c>
       <c r="I3" s="8">
-        <f>SUM(C9:L9)+SUM(C13:L13)-F3</f>
-        <v>2795271.9057673095</v>
-      </c>
-    </row>
-    <row r="4" spans="2:12" x14ac:dyDescent="0.35">
+        <f t="shared" ref="I3:I4" si="0">SUM($C$9:$L$9)-F3</f>
+        <v>1503542.1213406175</v>
+      </c>
+      <c r="K3" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="L3" s="8">
+        <f t="shared" ref="L3:L4" si="1">SUM($C$9:$L$9)+SUM($C$13:$G$13)-F3</f>
+        <v>2828158.13439776</v>
+      </c>
+      <c r="N3" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="O3" s="8">
+        <f>SUM($C$9:$L$9)+SUM($C$13:$L$13)-F3</f>
+        <v>3729669.5354062933</v>
+      </c>
+    </row>
+    <row r="4" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B4" t="s">
         <v>45</v>
       </c>
@@ -1728,11 +1779,25 @@
         <v>50</v>
       </c>
       <c r="I4" s="8">
-        <f>SUM(C9:L9)+SUM(C13:L13)-F4</f>
-        <v>1325271.9057673095</v>
-      </c>
-    </row>
-    <row r="7" spans="2:12" x14ac:dyDescent="0.35">
+        <f t="shared" si="0"/>
+        <v>33542.121340617537</v>
+      </c>
+      <c r="K4" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L4" s="8">
+        <f t="shared" si="1"/>
+        <v>1358158.13439776</v>
+      </c>
+      <c r="N4" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="O4" s="8">
+        <f>SUM($C$9:$L$9)+SUM($C$13:$L$13)-F4</f>
+        <v>2259669.5354062933</v>
+      </c>
+    </row>
+    <row r="7" spans="2:15" x14ac:dyDescent="0.35">
       <c r="C7" s="16" t="s">
         <v>47</v>
       </c>
@@ -1746,7 +1811,7 @@
       <c r="K7" s="16"/>
       <c r="L7" s="16"/>
     </row>
-    <row r="8" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="8" spans="2:15" x14ac:dyDescent="0.35">
       <c r="C8">
         <v>1</v>
       </c>
@@ -1778,49 +1843,49 @@
         <v>10</v>
       </c>
     </row>
-    <row r="9" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="9" spans="2:15" x14ac:dyDescent="0.35">
       <c r="C9" s="5">
-        <f t="shared" ref="C9:L9" si="0">$C$4/((1+$C$3)^C8)</f>
-        <v>651129.09090909082</v>
+        <f t="shared" ref="C9:L9" si="2">$C$4/((1+$C$3)^C8)</f>
+        <v>663187.03703703696</v>
       </c>
       <c r="D9" s="5">
-        <f t="shared" si="0"/>
-        <v>591935.5371900826</v>
+        <f t="shared" si="2"/>
+        <v>614062.07133058982</v>
       </c>
       <c r="E9" s="5">
-        <f t="shared" si="0"/>
-        <v>538123.2156273477</v>
+        <f t="shared" si="2"/>
+        <v>568575.99197276833</v>
       </c>
       <c r="F9" s="5">
-        <f t="shared" si="0"/>
-        <v>489202.92329758883</v>
+        <f t="shared" si="2"/>
+        <v>526459.25182663731</v>
       </c>
       <c r="G9" s="5">
-        <f t="shared" si="0"/>
-        <v>444729.93027053529</v>
+        <f t="shared" si="2"/>
+        <v>487462.27020984935</v>
       </c>
       <c r="H9" s="5">
-        <f t="shared" si="0"/>
-        <v>404299.93660957745</v>
+        <f t="shared" si="2"/>
+        <v>451353.95389800856</v>
       </c>
       <c r="I9" s="5">
-        <f t="shared" si="0"/>
-        <v>367545.39691779763</v>
+        <f t="shared" si="2"/>
+        <v>417920.32768334128</v>
       </c>
       <c r="J9" s="5">
-        <f t="shared" si="0"/>
-        <v>334132.1790161797</v>
+        <f t="shared" si="2"/>
+        <v>386963.26637346414</v>
       </c>
       <c r="K9" s="5">
-        <f t="shared" si="0"/>
-        <v>303756.52637834515</v>
+        <f t="shared" si="2"/>
+        <v>358299.32071617048</v>
       </c>
       <c r="L9" s="5">
-        <f t="shared" si="0"/>
-        <v>276142.2967075865</v>
-      </c>
-    </row>
-    <row r="12" spans="2:12" x14ac:dyDescent="0.35">
+        <f t="shared" si="2"/>
+        <v>331758.63029275043</v>
+      </c>
+    </row>
+    <row r="12" spans="2:15" x14ac:dyDescent="0.35">
       <c r="C12">
         <v>11</v>
       </c>
@@ -1852,51 +1917,54 @@
         <v>20</v>
       </c>
     </row>
-    <row r="13" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="13" spans="2:15" x14ac:dyDescent="0.35">
       <c r="C13" s="5">
-        <f t="shared" ref="C13:L13" si="1">$C$4/((1+$C$3)^C12)</f>
-        <v>251038.4515523513</v>
+        <f t="shared" ref="C13:L13" si="3">$C$4/((1+$C$3)^C12)</f>
+        <v>307183.91693773185</v>
       </c>
       <c r="D13" s="5">
-        <f t="shared" si="1"/>
-        <v>228216.77413850121</v>
+        <f t="shared" si="3"/>
+        <v>284429.5527201221</v>
       </c>
       <c r="E13" s="5">
-        <f t="shared" si="1"/>
-        <v>207469.79467136471</v>
+        <f t="shared" si="3"/>
+        <v>263360.69696307601</v>
       </c>
       <c r="F13" s="5">
-        <f t="shared" si="1"/>
-        <v>188608.90424669517</v>
+        <f t="shared" si="3"/>
+        <v>243852.49718803327</v>
       </c>
       <c r="G13" s="5">
-        <f t="shared" si="1"/>
-        <v>171462.64022426834</v>
+        <f t="shared" si="3"/>
+        <v>225789.34924817894</v>
       </c>
       <c r="H13" s="5">
-        <f t="shared" si="1"/>
-        <v>155875.12747660757</v>
+        <f t="shared" si="3"/>
+        <v>209064.21226683239</v>
       </c>
       <c r="I13" s="5">
-        <f t="shared" si="1"/>
-        <v>141704.66134237053</v>
+        <f t="shared" si="3"/>
+        <v>193577.97432114108</v>
       </c>
       <c r="J13" s="5">
-        <f t="shared" si="1"/>
-        <v>128822.41940215501</v>
+        <f t="shared" si="3"/>
+        <v>179238.86511216764</v>
       </c>
       <c r="K13" s="5">
-        <f t="shared" si="1"/>
-        <v>117111.29036559543</v>
+        <f t="shared" si="3"/>
+        <v>165961.91214089596</v>
       </c>
       <c r="L13" s="5">
-        <f t="shared" si="1"/>
-        <v>106464.80942326858</v>
+        <f t="shared" si="3"/>
+        <v>153668.43716749627</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="1">
+  <mergeCells count="4">
     <mergeCell ref="C7:L7"/>
+    <mergeCell ref="H1:I1"/>
+    <mergeCell ref="K1:L1"/>
+    <mergeCell ref="N1:O1"/>
   </mergeCells>
   <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1905,13 +1973,27 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BE8641AB-FA05-4689-970F-41940E5E4D56}">
-  <dimension ref="B2:V19"/>
+  <dimension ref="B1:V19"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="15.36328125" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="11.26953125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
+    <row r="1" spans="2:22" x14ac:dyDescent="0.35">
+      <c r="E1" s="16" t="s">
+        <v>72</v>
+      </c>
+      <c r="F1" s="16"/>
+      <c r="H1" s="16" t="s">
+        <v>73</v>
+      </c>
+      <c r="I1" s="16"/>
+      <c r="K1" s="16" t="s">
+        <v>71</v>
+      </c>
+      <c r="L1" s="16"/>
+    </row>
     <row r="2" spans="2:22" x14ac:dyDescent="0.35">
       <c r="B2" t="s">
         <v>45</v>
@@ -1924,6 +2006,20 @@
         <v>51</v>
       </c>
       <c r="F2" s="11">
+        <f>IRR(B9:L9)</f>
+        <v>0.14583203543754997</v>
+      </c>
+      <c r="H2" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="I2" s="11">
+        <f>IRR(B9:Q9)</f>
+        <v>0.17964512172791269</v>
+      </c>
+      <c r="K2" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="L2" s="11">
         <f>IRR(B9:V9)</f>
         <v>0.19005510390504865</v>
       </c>
@@ -1934,6 +2030,20 @@
         <v>55</v>
       </c>
       <c r="F3" s="11">
+        <f>IRR(B14:L14)</f>
+        <v>0.17284089361257693</v>
+      </c>
+      <c r="H3" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="I3" s="11">
+        <f>IRR(B14:Q14)</f>
+        <v>0.20338439889657356</v>
+      </c>
+      <c r="K3" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="L3" s="11">
         <f>IRR(B14:V14)</f>
         <v>0.21226254296401237</v>
       </c>
@@ -1943,6 +2053,20 @@
         <v>56</v>
       </c>
       <c r="F4" s="11">
+        <f>IRR(B19:L19)</f>
+        <v>8.1555704598693213E-2</v>
+      </c>
+      <c r="H4" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="I4" s="11">
+        <f>IRR(B19:Q19)</f>
+        <v>0.12413179874637659</v>
+      </c>
+      <c r="K4" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="L4" s="11">
         <f>IRR(B19:V19)</f>
         <v>0.13895488560750513</v>
       </c>
@@ -2443,10 +2567,13 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="3">
+  <mergeCells count="6">
     <mergeCell ref="C7:L7"/>
     <mergeCell ref="C12:L12"/>
     <mergeCell ref="C17:L17"/>
+    <mergeCell ref="E1:F1"/>
+    <mergeCell ref="H1:I1"/>
+    <mergeCell ref="K1:L1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -2591,7 +2718,7 @@
         <v>-3001370.9090909092</v>
       </c>
       <c r="D9" s="5">
-        <f t="shared" ref="C9:L9" si="1">$C$4/((1+$C$3)^D8)+C9</f>
+        <f t="shared" ref="D9:L9" si="1">$C$4/((1+$C$3)^D8)+C9</f>
         <v>-2409435.3719008267</v>
       </c>
       <c r="E9" s="5">

</xml_diff>